<commit_message>
Scrub legacy header remnants from the report template
</commit_message>
<xml_diff>
--- a/template/report_template.xlsx
+++ b/template/report_template.xlsx
@@ -1067,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AD1045"/>
+  <dimension ref="A2:AD1045"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="2.09765625" customWidth="1" style="56" min="1" max="1"/>
@@ -1103,7 +1103,6 @@
     <col width="11.69921875" customWidth="1" style="56" min="40" max="40"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="24.9" customHeight="1" s="56">
       <c r="B2" s="55" t="inlineStr">
         <is>
@@ -1112,11 +1111,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-14, HW Team</t>
-        </is>
-      </c>
+      <c r="B3" s="8" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1" s="56" thickBot="1">
       <c r="D4" s="63" t="n"/>
@@ -1130,85 +1125,85 @@
       </c>
       <c r="C5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-14 DUT#1</t>
+          <t>DUT#1</t>
         </is>
       </c>
       <c r="D5" s="58" t="n"/>
       <c r="E5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#2</t>
+          <t>DUT#2</t>
         </is>
       </c>
       <c r="F5" s="58" t="n"/>
       <c r="G5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#3</t>
+          <t>DUT#3</t>
         </is>
       </c>
       <c r="H5" s="58" t="n"/>
       <c r="I5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#4</t>
+          <t>DUT#4</t>
         </is>
       </c>
       <c r="J5" s="58" t="n"/>
       <c r="K5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#5</t>
+          <t>DUT#5</t>
         </is>
       </c>
       <c r="L5" s="58" t="n"/>
       <c r="M5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#6</t>
+          <t>DUT#6</t>
         </is>
       </c>
       <c r="N5" s="58" t="n"/>
       <c r="O5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#7</t>
+          <t>DUT#7</t>
         </is>
       </c>
       <c r="P5" s="58" t="n"/>
       <c r="Q5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#8</t>
+          <t>DUT#8</t>
         </is>
       </c>
       <c r="R5" s="58" t="n"/>
       <c r="S5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#9</t>
+          <t>DUT#9</t>
         </is>
       </c>
       <c r="T5" s="58" t="n"/>
       <c r="U5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#10</t>
+          <t>DUT#10</t>
         </is>
       </c>
       <c r="V5" s="58" t="n"/>
       <c r="W5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#11</t>
+          <t>DUT#11</t>
         </is>
       </c>
       <c r="X5" s="58" t="n"/>
       <c r="Y5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#12</t>
+          <t>DUT#12</t>
         </is>
       </c>
       <c r="Z5" s="58" t="n"/>
       <c r="AA5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#13</t>
+          <t>DUT#13</t>
         </is>
       </c>
       <c r="AB5" s="58" t="n"/>
       <c r="AC5" s="57" t="inlineStr">
         <is>
-          <t>2026-07-15 DUT#14</t>
+          <t>DUT#14</t>
         </is>
       </c>
       <c r="AD5" s="58" t="n"/>

</xml_diff>